<commit_message>
Update index: 16770 → 16900 [scan complete 03-08-2026]
Scanned addresses 16770-16899 in Jerusalem. Found 4 businesses:
- שנקולבסקי זכריה (עו"ד) - משעול המגלית 4
- איילת אביגדור-רפואה סינית - משעול המגלית 7
- אליספור דוד (קבלן בניין) - משפט דרייפוס 15
- בראשית מקיטן יעקב (תיווך) - משפט דרייפוס 4
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:03-08-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:03-08-2026.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כתובות שנסרקו" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="דוח עסקים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,16 +29,17 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="000563C1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -56,11 +56,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -82,65 +82,21 @@
         <color rgb="001F4E79"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="001F4E79"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="001F4E79"/>
-      </right>
-      <top style="thin">
-        <color rgb="001F4E79"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="001F4E79"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001F4E79"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="001F4E79"/>
-      </right>
-      <top style="thin">
-        <color rgb="001F4E79"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001F4E79"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -506,13 +462,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
@@ -555,111 +511,121 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>לא נמצאו עסקים בכתובות שנסרקו</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="4" t="n"/>
+          <t>שנקולבסקי זכריה (עו"ד)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>משעול המגלית 4, ירושלים</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>עורכי דין</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C041340746C5E4A140611/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>כתובת שנסרקה</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>ממצאים</t>
-        </is>
-      </c>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>איילת אביגדור-רפואה סינית</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>משעול המגלית 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>רפואה סינית</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80097769/40030001/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>משעול הדקלים 9, ירושלים</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>לא נמצאו עסקים</t>
-        </is>
-      </c>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>אליספור דוד</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>משפט דרייפוס 15, ירושלים</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>קבלני בניין</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/5905620/43470/</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>משעול ההדס 1, ירושלים</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>לא נמצאו עסקים</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>משעול ההדס 10, ירושלים</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>לא נמצאו עסקים</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>משעול ההדס 11, ירושלים</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>לא נמצאו עסקים</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>משעול ההדס 12, ירושלים</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>לא נמצאו עסקים</t>
-        </is>
-      </c>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>"בראשית" - מקיטן יעקב</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>משפט דרייפוס 4, ירושלים</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>תיווך נדל"ן</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/26778050/32970/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>